<commit_message>
[skip social] Complete existing business plans and uneven payback
</commit_message>
<xml_diff>
--- a/public/downloads/coffee-shop-business-plan-template.xlsx
+++ b/public/downloads/coffee-shop-business-plan-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Outline" sheetId="1" r:id="R4ce3ad2f776e4295"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Model" sheetId="2" r:id="R7a830043604c4b0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Outline" sheetId="1" r:id="Rc98822d5b3594437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Model" sheetId="2" r:id="R88410f4e8cb5464f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -774,7 +774,7 @@
         <x:v>Monthly orders</x:v>
       </x:c>
       <x:c r="B13" s="10" t="n">
-        <x:f>B6*B7</x:f>
+        <x:f>IF(COUNT(B6:B7)=2,B6*B7,"n.a.")</x:f>
         <x:v>2080</x:v>
       </x:c>
       <x:c r="C13" s="1"/>
@@ -786,7 +786,7 @@
         <x:v>Monthly sales USD</x:v>
       </x:c>
       <x:c r="B14" s="11" t="n">
-        <x:f>B13*B8</x:f>
+        <x:f>IF(AND(ISNUMBER(B13),ISNUMBER(B8)),B13*B8,"n.a.")</x:f>
         <x:v>24960</x:v>
       </x:c>
       <x:c r="C14" s="1"/>
@@ -798,7 +798,7 @@
         <x:v>Contribution per order USD</x:v>
       </x:c>
       <x:c r="B15" s="11" t="n">
-        <x:f>B8-B9</x:f>
+        <x:f>IF(COUNT(B8:B9)=2,B8-B9,"n.a.")</x:f>
         <x:v>7.5</x:v>
       </x:c>
       <x:c r="C15" s="1"/>
@@ -810,7 +810,7 @@
         <x:v>Monthly contribution USD</x:v>
       </x:c>
       <x:c r="B16" s="11" t="n">
-        <x:f>B13*B15</x:f>
+        <x:f>IF(AND(ISNUMBER(B13),ISNUMBER(B15)),B13*B15,"n.a.")</x:f>
         <x:v>15600</x:v>
       </x:c>
       <x:c r="C16" s="1"/>
@@ -822,7 +822,7 @@
         <x:v>Operating result USD</x:v>
       </x:c>
       <x:c r="B17" s="11" t="n">
-        <x:f>B16-B10</x:f>
+        <x:f>IF(AND(ISNUMBER(B16),ISNUMBER(B10)),B16-B10,"n.a.")</x:f>
         <x:v>600</x:v>
       </x:c>
       <x:c r="C17" s="1"/>
@@ -834,7 +834,7 @@
         <x:v>Break-even monthly orders</x:v>
       </x:c>
       <x:c r="B18" s="10" t="n">
-        <x:f>IFERROR(ROUNDUP(B10/B15,0),0)</x:f>
+        <x:f>IF(AND(ISNUMBER(B10),ISNUMBER(B15)),IF(B15&gt;0,ROUNDUP(B10/B15,0),"Not possible"),"n.a.")</x:f>
         <x:v>2000</x:v>
       </x:c>
       <x:c r="C18" s="1"/>
@@ -846,7 +846,7 @@
         <x:v>Break-even daily orders, rounded up</x:v>
       </x:c>
       <x:c r="B19" s="10" t="n">
-        <x:f>IFERROR(ROUNDUP(B18/B7,0),0)</x:f>
+        <x:f>IF(AND(ISNUMBER(B18),ISNUMBER(B7)),IF(B7&gt;0,ROUNDUP(B18/B7,0),"No trading days"),"n.a.")</x:f>
         <x:v>77</x:v>
       </x:c>
       <x:c r="C19" s="1"/>
@@ -858,7 +858,7 @@
         <x:v>Opening cash plus reserve USD</x:v>
       </x:c>
       <x:c r="B20" s="12" t="n">
-        <x:f>B11+B12</x:f>
+        <x:f>IF(COUNT(B11:B12)=2,SUM(B11:B12),"n.a.")</x:f>
         <x:v>50000</x:v>
       </x:c>
       <x:c r="C20" s="1"/>

</xml_diff>

<commit_message>
[skip social] Complete existing business plans and uneven payback (#176)
</commit_message>
<xml_diff>
--- a/public/downloads/coffee-shop-business-plan-template.xlsx
+++ b/public/downloads/coffee-shop-business-plan-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Outline" sheetId="1" r:id="R4ce3ad2f776e4295"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Model" sheetId="2" r:id="R7a830043604c4b0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Outline" sheetId="1" r:id="Rc98822d5b3594437"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Model" sheetId="2" r:id="R88410f4e8cb5464f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -774,7 +774,7 @@
         <x:v>Monthly orders</x:v>
       </x:c>
       <x:c r="B13" s="10" t="n">
-        <x:f>B6*B7</x:f>
+        <x:f>IF(COUNT(B6:B7)=2,B6*B7,"n.a.")</x:f>
         <x:v>2080</x:v>
       </x:c>
       <x:c r="C13" s="1"/>
@@ -786,7 +786,7 @@
         <x:v>Monthly sales USD</x:v>
       </x:c>
       <x:c r="B14" s="11" t="n">
-        <x:f>B13*B8</x:f>
+        <x:f>IF(AND(ISNUMBER(B13),ISNUMBER(B8)),B13*B8,"n.a.")</x:f>
         <x:v>24960</x:v>
       </x:c>
       <x:c r="C14" s="1"/>
@@ -798,7 +798,7 @@
         <x:v>Contribution per order USD</x:v>
       </x:c>
       <x:c r="B15" s="11" t="n">
-        <x:f>B8-B9</x:f>
+        <x:f>IF(COUNT(B8:B9)=2,B8-B9,"n.a.")</x:f>
         <x:v>7.5</x:v>
       </x:c>
       <x:c r="C15" s="1"/>
@@ -810,7 +810,7 @@
         <x:v>Monthly contribution USD</x:v>
       </x:c>
       <x:c r="B16" s="11" t="n">
-        <x:f>B13*B15</x:f>
+        <x:f>IF(AND(ISNUMBER(B13),ISNUMBER(B15)),B13*B15,"n.a.")</x:f>
         <x:v>15600</x:v>
       </x:c>
       <x:c r="C16" s="1"/>
@@ -822,7 +822,7 @@
         <x:v>Operating result USD</x:v>
       </x:c>
       <x:c r="B17" s="11" t="n">
-        <x:f>B16-B10</x:f>
+        <x:f>IF(AND(ISNUMBER(B16),ISNUMBER(B10)),B16-B10,"n.a.")</x:f>
         <x:v>600</x:v>
       </x:c>
       <x:c r="C17" s="1"/>
@@ -834,7 +834,7 @@
         <x:v>Break-even monthly orders</x:v>
       </x:c>
       <x:c r="B18" s="10" t="n">
-        <x:f>IFERROR(ROUNDUP(B10/B15,0),0)</x:f>
+        <x:f>IF(AND(ISNUMBER(B10),ISNUMBER(B15)),IF(B15&gt;0,ROUNDUP(B10/B15,0),"Not possible"),"n.a.")</x:f>
         <x:v>2000</x:v>
       </x:c>
       <x:c r="C18" s="1"/>
@@ -846,7 +846,7 @@
         <x:v>Break-even daily orders, rounded up</x:v>
       </x:c>
       <x:c r="B19" s="10" t="n">
-        <x:f>IFERROR(ROUNDUP(B18/B7,0),0)</x:f>
+        <x:f>IF(AND(ISNUMBER(B18),ISNUMBER(B7)),IF(B7&gt;0,ROUNDUP(B18/B7,0),"No trading days"),"n.a.")</x:f>
         <x:v>77</x:v>
       </x:c>
       <x:c r="C19" s="1"/>
@@ -858,7 +858,7 @@
         <x:v>Opening cash plus reserve USD</x:v>
       </x:c>
       <x:c r="B20" s="12" t="n">
-        <x:f>B11+B12</x:f>
+        <x:f>IF(COUNT(B11:B12)=2,SUM(B11:B12),"n.a.")</x:f>
         <x:v>50000</x:v>
       </x:c>
       <x:c r="C20" s="1"/>

</xml_diff>